<commit_message>
fix: move Gemini OCR call to backend to prevent client API key error in Vercel deployment
</commit_message>
<xml_diff>
--- a/public/카드매출 취소신청서.xlsx
+++ b/public/카드매출 취소신청서.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ProjectCode\las-mgmt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C2F2C8D-CA50-4A75-A883-F9C8A7A04BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B4A842-6CA5-4E5C-98F5-8C2BDE2AA8E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19785" yWindow="1665" windowWidth="16635" windowHeight="18825" xr2:uid="{D26891C3-CEC8-473A-A4F6-8C804C8C96AC}"/>
+    <workbookView xWindow="1965" yWindow="435" windowWidth="13440" windowHeight="20250" xr2:uid="{D26891C3-CEC8-473A-A4F6-8C804C8C96AC}"/>
   </bookViews>
   <sheets>
     <sheet name="보고서" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">보고서!$A$2:$E$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">보고서!$B$2:$F$12</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>접수일자</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -128,6 +128,10 @@
   </si>
   <si>
     <t>카드매출 취소 신청서</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>에이멘에이 주식회사</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -138,7 +142,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="&quot;₩&quot;#,##0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,6 +183,15 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -280,7 +293,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -299,6 +312,12 @@
     <xf numFmtId="176" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -322,9 +341,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -643,155 +659,165 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="B1:F14"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.75" customWidth="1"/>
-    <col min="2" max="2" width="14.25" customWidth="1"/>
-    <col min="3" max="3" width="26.25" customWidth="1"/>
-    <col min="4" max="4" width="14.25" customWidth="1"/>
-    <col min="5" max="5" width="26.75" customWidth="1"/>
+    <col min="2" max="2" width="15.75" customWidth="1"/>
+    <col min="3" max="3" width="14.25" customWidth="1"/>
+    <col min="4" max="4" width="26.25" customWidth="1"/>
+    <col min="5" max="5" width="14.25" customWidth="1"/>
+    <col min="6" max="6" width="26.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="2:6" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-    </row>
-    <row r="2" spans="1:5" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="3" t="s">
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+    </row>
+    <row r="2" spans="2:6" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="4"/>
-    </row>
-    <row r="3" spans="1:5" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="2:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="1"/>
+      <c r="E3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="11"/>
-      <c r="B4" s="3" t="s">
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="2:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="13"/>
+      <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4"/>
+      <c r="E4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="1"/>
-    </row>
-    <row r="5" spans="1:5" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="12" t="s">
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="2:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="1"/>
+      <c r="E5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="4"/>
-    </row>
-    <row r="6" spans="1:5" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="12"/>
-      <c r="B6" s="3" t="s">
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6" spans="2:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="14"/>
+      <c r="C6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="5"/>
+      <c r="E6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="12"/>
-      <c r="B7" s="3" t="s">
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="2:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="14"/>
+      <c r="C7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="10"/>
-    </row>
-    <row r="8" spans="1:5" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="12"/>
-      <c r="B8" s="3" t="s">
+      <c r="D7" s="10"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="12"/>
+    </row>
+    <row r="8" spans="2:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="14"/>
+      <c r="C8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="1"/>
+      <c r="E8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:5" ht="171" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="2:6" ht="171" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="10"/>
-    </row>
-    <row r="10" spans="1:5" ht="276.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+      <c r="C9" s="10"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="12"/>
+    </row>
+    <row r="10" spans="2:6" ht="276.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="C10" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="10"/>
-    </row>
-    <row r="11" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="11" t="s">
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="12"/>
+    </row>
+    <row r="11" spans="2:6" ht="42.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="1"/>
+      <c r="E11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="12"/>
-      <c r="B12" s="3" t="s">
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" spans="2:6" ht="42.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="14"/>
+      <c r="C12" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="12"/>
+    </row>
+    <row r="14" spans="2:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A5:A8"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="C7:E7"/>
+  <mergeCells count="10">
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="B5:B8"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="D7:F7"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>